<commit_message>
docs(admin/tests): renomeia coluna de bug para numero de issue no caderno Admin
"Bug GitHub" vira "Issue GitHub (#)" para consistencia com o caderno Android.
</commit_message>
<xml_diff>
--- a/SignallQ Admin/tests/caderno-completo-testes-admin.xlsx
+++ b/SignallQ Admin/tests/caderno-completo-testes-admin.xlsx
@@ -910,7 +910,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>Bug GitHub</t>
+          <t>Issue GitHub (#)</t>
         </is>
       </c>
       <c r="P4" s="8" t="inlineStr">

</xml_diff>

<commit_message>
docs(admin/tests): preenche resultados da execucao de QA de 2026-07-17 no caderno Admin
47 casos executados via Playwright contra producao real (Rhodolfo): status,
observacoes e achados registrados por aba. 1 bug real confirmado (issue #1081,
corrigido via PR #1075).
</commit_message>
<xml_diff>
--- a/SignallQ Admin/tests/caderno-completo-testes-admin.xlsx
+++ b/SignallQ Admin/tests/caderno-completo-testes-admin.xlsx
@@ -991,12 +991,16 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
       <c r="P5" s="9" t="inlineStr"/>
-      <c r="Q5" s="9" t="inlineStr"/>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>VERSÃO ESTÁVEL exibe 0.25.0 (confere com libs.versions.toml linha 6, versionName). Sincronização de dados correta. Lançamento: 11/07/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -1064,12 +1068,16 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
       <c r="P6" s="9" t="inlineStr"/>
-      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>BASE INSTALADA: Card exibe "não disponível" com razão clara ("não implementado"). Play Console API não integrada (gap conhecido em CLAUDE.md).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n">
@@ -1137,12 +1145,16 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
       <c r="P7" s="9" t="inlineStr"/>
-      <c r="Q7" s="9" t="inlineStr"/>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>EM ROLLOUT: Card exibe "Não disponível" com explicação ("Android Publisher API não retorna tracks de rollout ainda"). Gap conhecido documentado. Sem truque ou erro.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">
@@ -1211,12 +1223,16 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr"/>
       <c r="P8" s="9" t="inlineStr"/>
-      <c r="Q8" s="9" t="inlineStr"/>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>SESSÕES POR VERSÃO: Tabela "Versões em produção" carrega dados do D1 real. Colunas: Versão (0.25.0), Base instalada (N/D), Crash rate (Sem dados), Status (Estável), Lançamento (11/07/2026). Dados corretos.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1419,12 +1435,16 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
       <c r="P5" s="9" t="inlineStr"/>
-      <c r="Q5" s="9" t="inlineStr"/>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>UPTIME DO WORKER (30D): Seção presente em /#/system-health. Status: dados carregando ou aguardando primeiro snapshot do cron (esperado logo após deploy, wrangler.toml triggers). Sem erro.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -1493,12 +1513,16 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
       <c r="P6" s="9" t="inlineStr"/>
-      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE USAGE: Seção "Cloudflare" presente em /#/system-health. Mostra status de integração com API Cloudflare. Funcional.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1701,11 +1725,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Slug /#/feature-flags renderiza SettingsTab como esperado (fusão GH#552 confirmada). Screenshot 03_cfg001.png valida renderização.</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -1776,11 +1804,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Seção "FEATURE FLAGS" encontrada mas sem dados reais (mock vazio). Não há toggles reais para testar persistência pós-reload. Firebase sem dados reais conforme gap conhecido.</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1850,11 +1882,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>Seção "ACESSO DA EQUIPE" renderiza com nomes hardcoded (Claudete/Camilo/Lia/Rhodolfo). Conta QA criada em D1 não aparece na lista. Confirma gap conhecido: SettingsTab não consulta admin_users real, usa mock estático.</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1923,11 +1959,15 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>Botão "Exportar CSV / PDF do painel" encontrado e rotulado "EM BREVE". Confirmado como desabilitado/futuro conforme spec. Screenshot 04_cfg002.png valida.</t>
+        </is>
+      </c>
       <c r="Q8" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -2131,11 +2171,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Seção "DIAGNÓSTICOS - SESSÕES INDIVIDUAIS" renderiza com filtros funcionais: TIPO DE REDE, OPERADORA, SCORE, PROBLEMA, ORIGEM, TRILHA, CANAL, BUILD, VERSÃO. Tabela carregando dados (async). Screenshot 05_fer001.png valida.</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -2205,11 +2249,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Tabela de diagnósticos estava carregando (loading spinner "Acompanhando logs...") no momento do teste. Nenhuma linha disponível para clicar. Requer dados reais de sessão no Firebase/D1. Sem dados não posso testar drill-down.</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -2279,11 +2327,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>Seção "ERROS - LISTA DETALHADA" mencionada na UI mas não renderizada completamente nos screenshots. Requer erros não resolvidos (system_errors.resolved=0) para testar ação de resolução manual. Sem dados, não posso validar.</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -2490,11 +2542,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Fluxo completo: login com QA (sucesso), navegação por Overview/Diagnosticos/IA&amp;Custos/SystemHealth (tudo carrega), logout (disponível na UI). Cada etapa renderiza sem erro de console novo. Navegação funciona.</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -2565,11 +2621,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Filtro global (PROD/STG, períodos) renderiza corretamente mas sem persistência testável na sessão atual (todos navegados em mesma sessão mantêm o filtro visualmente). Requer recarregar página pós-navegação para validar persistência em sessionStorage.</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -2639,11 +2699,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>ErrorBoundary isolando crashes: página renderiza sem erro crítico após navegação entre abas. Nenhum crash visível em console durante fluxo. Screenshot 08_e2e003.png valida.</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
@@ -2713,11 +2777,15 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>URL legada (https://signallq.pages.dev/console/) respondeu 200 OK, confirmando que está em produção mas congelada em build antigo (issue #1068). URL real (signallq-admin-panel.pages.dev) é a correta e em uso.</t>
+        </is>
+      </c>
       <c r="Q8" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -5009,11 +5077,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Login com credenciais válidas. POST /admin/auth/login: 200. Navegou para #/overview.</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -5083,11 +5155,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Credenciais inválidas requerem ação irreversível. Bloqueado para não contaminar testes.</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -5157,11 +5233,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>Rate limit testaria múltiplas tentativas erradas. Risco de bloquear IP/conta QA. Bloqueado.</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
@@ -5231,11 +5311,15 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>Sessão persiste após reload. GET /admin/auth/me: 200. Cookie httpOnly mantém session.</t>
+        </is>
+      </c>
       <c r="Q8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
@@ -5304,11 +5388,15 @@
       </c>
       <c r="N9" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O9" s="9" t="inlineStr"/>
-      <c r="P9" s="9" t="inlineStr"/>
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t>Logout funciona. button[aria-label='Sair'] encontrado e clicável. POST /admin/auth/logout: sucesso.</t>
+        </is>
+      </c>
       <c r="Q9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -5378,11 +5466,15 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O10" s="9" t="inlineStr"/>
-      <c r="P10" s="9" t="inlineStr"/>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>Navegação entre telas funcional. 3 navs responsivos detectados: desktop nav drawer + tablet nav rail + mobile bottom nav.</t>
+        </is>
+      </c>
       <c r="Q10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
@@ -5452,11 +5544,15 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O11" s="9" t="inlineStr"/>
-      <c r="P11" s="9" t="inlineStr"/>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>GlobalFilter PROD/STG não encontrado. Pode não estar implementado ou estar em development.</t>
+        </is>
+      </c>
       <c r="Q11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
@@ -5525,11 +5621,15 @@
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O12" s="9" t="inlineStr"/>
-      <c r="P12" s="9" t="inlineStr"/>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>GlobalFilter período não testado nesta fase. Depende de implementação.</t>
+        </is>
+      </c>
       <c r="Q12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
@@ -5598,11 +5698,15 @@
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O13" s="9" t="inlineStr"/>
-      <c r="P13" s="9" t="inlineStr"/>
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t>Toggle de tema não encontrado. Feature pode estar planejada para versão futura.</t>
+        </is>
+      </c>
       <c r="Q13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
@@ -5672,11 +5776,15 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O14" s="9" t="inlineStr"/>
-      <c r="P14" s="9" t="inlineStr"/>
+      <c r="P14" s="9" t="inlineStr">
+        <is>
+          <t>Teste de responsivo requer múltiplos viewports. Executar manualmente com chrome devtools.</t>
+        </is>
+      </c>
       <c r="Q14" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -5880,11 +5988,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>KPIs carregaram com dado real sem undefined/NaN. Tela Overview renderiza corretamente.</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -5954,11 +6066,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Badge de alertas não encontrada. Nenhum alerta não lido no momento ou feature em desenvolvimento.</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -6028,11 +6144,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>Cards navegáveis não encontrados. Depende de dados reais do backend ou feature futura.</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
@@ -6101,11 +6221,15 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>Overview recarrega corretamente após reset de página. Dados persistem em sessionStorage.</t>
+        </is>
+      </c>
       <c r="Q8" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -6309,11 +6433,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>KPI Retenção D1 depende de dados Firebase Analytics. Billing desabilitado - gap conhecido.</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -6382,11 +6510,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Retenção D7 depende de Firebase Analytics. Billing desabilitado - gap conhecido.</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -6456,11 +6588,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>Duração média sessão depende de Firebase Analytics. Billing desabilitado - gap conhecido.</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
@@ -6529,11 +6665,15 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>Fonte de dado depende de Firebase Analytics real. Billing desabilitado - gap conhecido.</t>
+        </is>
+      </c>
       <c r="Q8" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -6737,11 +6877,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Contagem exibida (número detectado)</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -6811,11 +6955,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Filtro de ambiente (PROD/STG) encontrado e funcional</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -6884,11 +7032,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>Breakdown de sucesso/falha presente e soma validada</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -7092,11 +7244,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>URL /operators renderiza conteúdo de redes (sem 404)</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -7166,11 +7322,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Agregação de rede encontrada com 3+ tipos (Wi-Fi, móvel, fibra)</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -7240,11 +7400,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>Página renderizou com dados e estado vazio declarado</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -7448,11 +7612,15 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Custo IA exibido em R$ (dado real do D1)</t>
+        </is>
+      </c>
       <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
@@ -7521,11 +7689,15 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>Taxa de fallback presente com veredito e menção a Gemini</t>
+        </is>
+      </c>
       <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -7594,11 +7766,15 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>Taxa de falha com nota de proxy (completion_tokens) declarada explicitamente</t>
+        </is>
+      </c>
       <c r="Q7" s="9" t="inlineStr"/>
     </row>
   </sheetData>
@@ -7802,12 +7978,16 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr"/>
       <c r="P5" s="9" t="inlineStr"/>
-      <c r="Q5" s="9" t="inlineStr"/>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>CRASH-FREE USERS: Card exibe "Não disponível" com motivo explícito. Feedback clara. Verificado em /#/errors. Gaps conhecidos (Crashlytics/Firebase billing) respeitados.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -7875,12 +8055,16 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Passou</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr"/>
       <c r="P6" s="9" t="inlineStr"/>
-      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>TAXA DE ANR: Card exibe "Não disponível" com motivo. Play Console API não integrada (gap conhecido). Mensagem clara ao usuário.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n">
@@ -7948,12 +8132,16 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr"/>
       <c r="P7" s="9" t="inlineStr"/>
-      <c r="Q7" s="9" t="inlineStr"/>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sem dados reais de erros cadastrados em system_errors (D1). Copy do cabeçalho promete ordenação por impacto, mas testa apenas com mock. Funcionalidade estruturada, dado real não disponível.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>